<commit_message>
Add actual-source work assignment and template-matched settlements
</commit_message>
<xml_diff>
--- a/settlement-domestic-template.xlsx
+++ b/settlement-domestic-template.xlsx
@@ -32,6 +32,8 @@
     <definedName name="SD">'[3]KVC_출고의뢰 (2)'!$C$19</definedName>
     <definedName name="SE">'[4]KVC_출고의뢰 (2)'!$C$19</definedName>
     <definedName name="출고의뢰">'[3]KVC_출고의뢰 (2)'!$C$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'S.T'!$B$1:$K$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'S.T (2)'!$B$1:$K$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -6250,8 +6252,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A0B5D11-80F4-4002-A30B-B2D9878D47EF}">
   <sheetPr>
     <tabColor indexed="18"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J38"/>
+  <dimension ref="B1:K38"/>
   <sheetFormatPr defaultColWidth="9.75" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -6263,7 +6266,8 @@
     <col min="7" max="8" width="15.58203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.58203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="30.58203125" style="1" customWidth="1"/>
-    <col min="11" max="16" width="9.75" style="1" customWidth="1"/>
+    <col min="11" max="11" width="4" style="1" customWidth="1"/>
+    <col min="12" max="16" width="9.75" style="1" customWidth="1"/>
     <col min="17" max="20" width="9.75" style="1"/>
     <col min="21" max="37" width="9.75" style="1" customWidth="1"/>
     <col min="38" max="45" width="9.75" style="1"/>
@@ -6281,15 +6285,17 @@
       <c r="F2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="52" t="s">
-        <v>22</v>
+      <c r="G2" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">삼원스틸 주식회사</t>
+        </is>
       </c>
       <c r="H2" s="52"/>
       <c r="I2" s="22" t="s">
         <v>15</v>
       </c>
       <c r="J2" s="23">
-        <v>46240</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="33" customHeight="1">
@@ -6299,9 +6305,7 @@
       <c r="F3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="52" t="s">
-        <v>23</v>
-      </c>
+      <c r="G3" s="52"/>
       <c r="H3" s="52"/>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -6313,9 +6317,7 @@
       <c r="F4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="52" t="s">
-        <v>24</v>
-      </c>
+      <c r="G4" s="52"/>
       <c r="H4" s="52"/>
       <c r="I4" s="52"/>
       <c r="J4" s="52"/>
@@ -6329,9 +6331,7 @@
       <c r="F5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="52" t="s">
-        <v>25</v>
-      </c>
+      <c r="G5" s="52"/>
       <c r="H5" s="52"/>
       <c r="I5" s="52"/>
       <c r="J5" s="52"/>
@@ -6343,8 +6343,10 @@
       <c r="F6" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="52">
-        <v>8920</v>
+      <c r="G6" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">260724-7</t>
+        </is>
       </c>
       <c r="H6" s="52"/>
       <c r="I6" s="52"/>
@@ -6401,41 +6403,66 @@
       <c r="J9" s="32" t="s">
         <v>6</v>
       </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사진</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="2:10" ht="24" customHeight="1">
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">254SMO SOLID</t>
+        </is>
+      </c>
+      <c r="C10" s="13">
+        <v>2777</v>
+      </c>
       <c r="D10" s="12"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 925 · VS</t>
+        </is>
+      </c>
+      <c r="G10" s="15">
+        <v>352</v>
+      </c>
       <c r="H10" s="16"/>
-      <c r="I10" s="15"/>
+      <c r="I10" s="15">
+        <v>0</v>
+      </c>
       <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="2:10" ht="24" customHeight="1">
-      <c r="B11" s="12" t="s">
-        <v>26</v>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C-276 SOLID</t>
+        </is>
       </c>
       <c r="C11" s="13">
-        <v>4290</v>
+        <v>1094</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="12" t="str">
-        <f>B11</f>
-        <v>Ti 64 TUR</v>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 718 · VS</t>
+        </is>
       </c>
       <c r="G11" s="15">
-        <v>4125</v>
+        <v>742</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11" s="16">
-        <f>G11*H11</f>
         <v>0</v>
       </c>
-      <c r="J11" s="37" t="s">
-        <v>33</v>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●</t>
+        </is>
       </c>
     </row>
     <row r="12" spans="2:10" ht="24" customHeight="1">
@@ -6443,63 +6470,100 @@
       <c r="C12" s="13"/>
       <c r="D12" s="12"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="12" t="s">
-        <v>32</v>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · 254 · SOLID</t>
+        </is>
       </c>
       <c r="G12" s="15">
-        <v>66</v>
+        <v>1277</v>
       </c>
       <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
+      <c r="I12" s="16">
+        <v>0</v>
+      </c>
       <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
     </row>
     <row r="13" spans="2:10" ht="24" customHeight="1">
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="12"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="12" t="s">
-        <v>27</v>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · 254 · AS</t>
+        </is>
       </c>
       <c r="G13" s="15">
-        <v>99</v>
+        <v>1200</v>
       </c>
       <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
+      <c r="I13" s="16">
+        <v>0</v>
+      </c>
       <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
     </row>
     <row r="14" spans="2:10" ht="24" customHeight="1">
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="12"/>
       <c r="E14" s="11"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="15"/>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · sus 304 · SOLID</t>
+        </is>
+      </c>
+      <c r="G14" s="15">
+        <v>95</v>
+      </c>
       <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
       <c r="J14" s="37"/>
+      <c r="K14" s="37"/>
     </row>
     <row r="15" spans="2:10" ht="24" customHeight="1">
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="12"/>
       <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="15"/>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 718 · AS</t>
+        </is>
+      </c>
+      <c r="G15" s="15">
+        <v>200</v>
+      </c>
       <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
+      <c r="I15" s="16">
+        <v>0</v>
+      </c>
       <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
     </row>
     <row r="16" spans="2:10" ht="24" customHeight="1">
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="12"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="15"/>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOSS · 작업중 로스</t>
+        </is>
+      </c>
+      <c r="G16" s="15">
+        <v>5</v>
+      </c>
       <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
+      <c r="I16" s="16">
+        <v>0</v>
+      </c>
       <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="2:10" ht="24" customHeight="1">
       <c r="B17" s="12"/>
@@ -6511,6 +6575,7 @@
       <c r="H17" s="26"/>
       <c r="I17" s="26"/>
       <c r="J17" s="37"/>
+      <c r="K17"/>
     </row>
     <row r="18" spans="2:10" ht="24" customHeight="1">
       <c r="B18" s="12"/>
@@ -6522,6 +6587,7 @@
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="37"/>
+      <c r="K18"/>
     </row>
     <row r="19" spans="2:10" ht="24" customHeight="1">
       <c r="B19" s="12"/>
@@ -6533,6 +6599,7 @@
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="37"/>
+      <c r="K19"/>
     </row>
     <row r="20" spans="2:10" ht="24" customHeight="1">
       <c r="B20" s="12"/>
@@ -6544,6 +6611,7 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="37"/>
+      <c r="K20"/>
     </row>
     <row r="21" spans="2:10" ht="24" customHeight="1">
       <c r="B21" s="12"/>
@@ -6555,6 +6623,7 @@
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="17"/>
+      <c r="K21"/>
     </row>
     <row r="22" spans="2:10" ht="24" customHeight="1">
       <c r="B22" s="12"/>
@@ -6566,6 +6635,7 @@
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
       <c r="J22" s="17"/>
+      <c r="K22"/>
     </row>
     <row r="23" spans="2:10" ht="24" customHeight="1">
       <c r="B23" s="12"/>
@@ -6577,6 +6647,7 @@
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
+      <c r="K23"/>
     </row>
     <row r="24" spans="2:10" ht="24" customHeight="1">
       <c r="B24" s="12"/>
@@ -6588,6 +6659,7 @@
       <c r="H24" s="26"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
+      <c r="K24"/>
     </row>
     <row r="25" spans="2:10" ht="24" customHeight="1">
       <c r="B25" s="12"/>
@@ -6599,6 +6671,7 @@
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
+      <c r="K25"/>
     </row>
     <row r="26" spans="2:10" ht="24" customHeight="1">
       <c r="B26" s="17"/>
@@ -6607,14 +6680,16 @@
       <c r="E26" s="11"/>
       <c r="F26" s="14"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15" t="s">
-        <v>13</v>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공급가액 :</t>
+        </is>
       </c>
       <c r="I26" s="15">
-        <f>SUM(I10:I25)</f>
         <v>0</v>
       </c>
       <c r="J26" s="17"/>
+      <c r="K26"/>
     </row>
     <row r="27" spans="2:10" ht="24" customHeight="1">
       <c r="B27" s="18"/>
@@ -6623,38 +6698,46 @@
       <c r="E27" s="11"/>
       <c r="F27" s="14"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15" t="s">
-        <v>14</v>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">부가세 :</t>
+        </is>
       </c>
       <c r="I27" s="15">
-        <f>I26*10%</f>
         <v>0</v>
       </c>
       <c r="J27" s="18"/>
+      <c r="K27"/>
     </row>
     <row r="28" spans="2:10" ht="24" customHeight="1">
-      <c r="B28" s="35" t="s">
-        <v>8</v>
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
       </c>
       <c r="C28" s="34">
-        <f>SUM(C10:C27)</f>
-        <v>4290</v>
+        <v>3871</v>
       </c>
       <c r="D28" s="34"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="32"/>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
       <c r="G28" s="19">
-        <f>SUM(G10:G27)</f>
-        <v>4290</v>
+        <v>3871</v>
       </c>
       <c r="H28" s="19"/>
-      <c r="I28" s="20" t="s">
-        <v>9</v>
+      <c r="I28" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total :</t>
+        </is>
       </c>
       <c r="J28" s="20">
-        <f>I26+I27</f>
         <v>0</v>
       </c>
+      <c r="K28"/>
     </row>
     <row r="29" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B29" s="9"/>
@@ -6666,10 +6749,13 @@
       <c r="H29" s="24"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
+      <c r="K29"/>
     </row>
     <row r="30" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B30" s="41" t="s">
-        <v>28</v>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">세금계산서 발행 요청일 : 2026-07-27</t>
+        </is>
       </c>
       <c r="C30" s="42"/>
       <c r="D30" s="42"/>
@@ -6681,9 +6767,14 @@
       <c r="J30" s="21" t="s">
         <v>10</v>
       </c>
+      <c r="K30"/>
     </row>
     <row r="31" spans="2:10" ht="45" customHeight="1">
-      <c r="B31" s="44"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">세금계산서 작성일자 : 2026-07-27</t>
+        </is>
+      </c>
       <c r="C31" s="45"/>
       <c r="D31" s="45"/>
       <c r="E31" s="45"/>
@@ -6693,9 +6784,14 @@
       <c r="J31" s="31" t="s">
         <v>11</v>
       </c>
+      <c r="K31"/>
     </row>
     <row r="32" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B32" s="47"/>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">발행 마감 : 오후 4시</t>
+        </is>
+      </c>
       <c r="C32" s="48"/>
       <c r="D32" s="48"/>
       <c r="E32" s="48"/>
@@ -6705,6 +6801,7 @@
       <c r="J32" s="8" t="s">
         <v>12</v>
       </c>
+      <c r="K32"/>
     </row>
     <row r="33" ht="16.5" customHeight="1"/>
     <row r="34" ht="16.5" customHeight="1"/>
@@ -6727,7 +6824,7 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.51181102362204722" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -6736,8 +6833,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F648DCA-04E3-49E1-80BE-BA0535619566}">
   <sheetPr>
     <tabColor indexed="18"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J38"/>
+  <dimension ref="B1:K38"/>
   <sheetFormatPr defaultColWidth="9.75" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -6749,7 +6847,8 @@
     <col min="7" max="8" width="15.58203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.58203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="30.58203125" style="1" customWidth="1"/>
-    <col min="11" max="16" width="9.75" style="1" customWidth="1"/>
+    <col min="11" max="11" width="4" style="1" customWidth="1"/>
+    <col min="12" max="16" width="9.75" style="1" customWidth="1"/>
     <col min="17" max="20" width="9.75" style="1"/>
     <col min="21" max="37" width="9.75" style="1" customWidth="1"/>
     <col min="38" max="45" width="9.75" style="1"/>
@@ -6767,15 +6866,17 @@
       <c r="F2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="52" t="s">
-        <v>22</v>
+      <c r="G2" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">삼원스틸 주식회사</t>
+        </is>
       </c>
       <c r="H2" s="52"/>
       <c r="I2" s="22" t="s">
         <v>15</v>
       </c>
       <c r="J2" s="23">
-        <v>46240</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="33" customHeight="1">
@@ -6785,9 +6886,7 @@
       <c r="F3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="52" t="s">
-        <v>23</v>
-      </c>
+      <c r="G3" s="52"/>
       <c r="H3" s="52"/>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -6799,9 +6898,7 @@
       <c r="F4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="52" t="s">
-        <v>24</v>
-      </c>
+      <c r="G4" s="52"/>
       <c r="H4" s="52"/>
       <c r="I4" s="52"/>
       <c r="J4" s="52"/>
@@ -6815,9 +6912,7 @@
       <c r="F5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="52" t="s">
-        <v>25</v>
-      </c>
+      <c r="G5" s="52"/>
       <c r="H5" s="52"/>
       <c r="I5" s="52"/>
       <c r="J5" s="52"/>
@@ -6829,8 +6924,10 @@
       <c r="F6" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="52">
-        <v>8920</v>
+      <c r="G6" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">260724-7</t>
+        </is>
       </c>
       <c r="H6" s="52"/>
       <c r="I6" s="52"/>
@@ -6887,134 +6984,179 @@
       <c r="J9" s="32" t="s">
         <v>6</v>
       </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사진</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="2:10" ht="24" customHeight="1">
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">254SMO SOLID</t>
+        </is>
+      </c>
+      <c r="C10" s="13">
+        <v>2777</v>
+      </c>
       <c r="D10" s="12"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 925 · VS</t>
+        </is>
+      </c>
+      <c r="G10" s="15">
+        <v>352</v>
+      </c>
       <c r="H10" s="16"/>
-      <c r="I10" s="15"/>
+      <c r="I10" s="15">
+        <v>0</v>
+      </c>
       <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="2:10" ht="24" customHeight="1">
-      <c r="B11" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="13"/>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C-276 SOLID</t>
+        </is>
+      </c>
+      <c r="C11" s="13">
+        <v>1094</v>
+      </c>
       <c r="D11" s="12"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 718 · VS</t>
+        </is>
+      </c>
+      <c r="G11" s="15">
+        <v>742</v>
+      </c>
       <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
+      <c r="I11" s="16">
+        <v>0</v>
+      </c>
       <c r="J11" s="37"/>
+      <c r="K11" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="2:10" ht="24" customHeight="1">
-      <c r="B12" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="13">
-        <v>5200</v>
-      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="12"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="12" t="str">
-        <f>B12</f>
-        <v>Ti 64 TUR</v>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · 254 · SOLID</t>
+        </is>
       </c>
       <c r="G12" s="15">
-        <v>5060</v>
-      </c>
-      <c r="H12" s="16">
-        <v>3000</v>
-      </c>
+        <v>1277</v>
+      </c>
+      <c r="H12" s="16"/>
       <c r="I12" s="16">
-        <f>G12*H12</f>
-        <v>15180000</v>
+        <v>0</v>
       </c>
       <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
     </row>
     <row r="13" spans="2:10" ht="24" customHeight="1">
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="12"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="12" t="s">
-        <v>31</v>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · 254 · AS</t>
+        </is>
       </c>
       <c r="G13" s="15">
-        <v>140</v>
+        <v>1200</v>
       </c>
       <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
+      <c r="I13" s="16">
+        <v>0</v>
+      </c>
       <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
     </row>
     <row r="14" spans="2:10" ht="24" customHeight="1">
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="12"/>
       <c r="E14" s="11"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="15"/>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STS · sus 304 · SOLID</t>
+        </is>
+      </c>
+      <c r="G14" s="15">
+        <v>95</v>
+      </c>
       <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
+      <c r="I14" s="26">
+        <v>0</v>
+      </c>
       <c r="J14" s="37"/>
+      <c r="K14" s="37"/>
     </row>
     <row r="15" spans="2:10" ht="24" customHeight="1">
-      <c r="B15" s="12" t="s">
-        <v>30</v>
-      </c>
+      <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="12"/>
       <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="15"/>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NI · IN 718 · AS</t>
+        </is>
+      </c>
+      <c r="G15" s="15">
+        <v>200</v>
+      </c>
       <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
+      <c r="I15" s="26">
+        <v>0</v>
+      </c>
       <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
     </row>
     <row r="16" spans="2:10" ht="24" customHeight="1">
-      <c r="B16" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="13">
-        <v>4290</v>
-      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
       <c r="D16" s="12"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="12" t="str">
-        <f>B16</f>
-        <v>Ti 64 TUR</v>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOSS · 작업중 로스</t>
+        </is>
       </c>
       <c r="G16" s="15">
-        <v>4191</v>
-      </c>
-      <c r="H16" s="16">
-        <v>1600</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="H16" s="16"/>
       <c r="I16" s="16">
-        <f>G16*H16</f>
-        <v>6705600</v>
+        <v>0</v>
       </c>
       <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="2:10" ht="24" customHeight="1">
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="12"/>
       <c r="E17" s="11"/>
-      <c r="F17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="15">
-        <v>99</v>
-      </c>
+      <c r="F17" s="12"/>
+      <c r="G17" s="15"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="37"/>
+      <c r="K17"/>
     </row>
     <row r="18" spans="2:10" ht="24" customHeight="1">
       <c r="B18" s="12"/>
@@ -7026,6 +7168,7 @@
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="37"/>
+      <c r="K18"/>
     </row>
     <row r="19" spans="2:10" ht="24" customHeight="1">
       <c r="B19" s="12"/>
@@ -7037,6 +7180,7 @@
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="37"/>
+      <c r="K19"/>
     </row>
     <row r="20" spans="2:10" ht="24" customHeight="1">
       <c r="B20" s="12"/>
@@ -7048,6 +7192,7 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="37"/>
+      <c r="K20"/>
     </row>
     <row r="21" spans="2:10" ht="24" customHeight="1">
       <c r="B21" s="12"/>
@@ -7059,6 +7204,7 @@
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="17"/>
+      <c r="K21"/>
     </row>
     <row r="22" spans="2:10" ht="24" customHeight="1">
       <c r="B22" s="12"/>
@@ -7070,6 +7216,7 @@
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
       <c r="J22" s="17"/>
+      <c r="K22"/>
     </row>
     <row r="23" spans="2:10" ht="24" customHeight="1">
       <c r="B23" s="12"/>
@@ -7081,6 +7228,7 @@
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
+      <c r="K23"/>
     </row>
     <row r="24" spans="2:10" ht="24" customHeight="1">
       <c r="B24" s="12"/>
@@ -7092,6 +7240,7 @@
       <c r="H24" s="26"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
+      <c r="K24"/>
     </row>
     <row r="25" spans="2:10" ht="24" customHeight="1">
       <c r="B25" s="12"/>
@@ -7103,6 +7252,7 @@
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
+      <c r="K25"/>
     </row>
     <row r="26" spans="2:10" ht="24" customHeight="1">
       <c r="B26" s="17"/>
@@ -7111,14 +7261,16 @@
       <c r="E26" s="11"/>
       <c r="F26" s="14"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15" t="s">
-        <v>13</v>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공급가액 :</t>
+        </is>
       </c>
       <c r="I26" s="15">
-        <f>SUM(I10:I25)</f>
-        <v>21885600</v>
+        <v>0</v>
       </c>
       <c r="J26" s="17"/>
+      <c r="K26"/>
     </row>
     <row r="27" spans="2:10" ht="24" customHeight="1">
       <c r="B27" s="18"/>
@@ -7127,38 +7279,46 @@
       <c r="E27" s="11"/>
       <c r="F27" s="14"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15" t="s">
-        <v>14</v>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">부가세 :</t>
+        </is>
       </c>
       <c r="I27" s="15">
-        <f>I26*10%</f>
-        <v>2188560</v>
+        <v>0</v>
       </c>
       <c r="J27" s="18"/>
+      <c r="K27"/>
     </row>
     <row r="28" spans="2:10" ht="24" customHeight="1">
-      <c r="B28" s="35" t="s">
-        <v>8</v>
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
       </c>
       <c r="C28" s="34">
-        <f>SUM(C10:C27)</f>
-        <v>9490</v>
+        <v>3871</v>
       </c>
       <c r="D28" s="34"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="32"/>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
       <c r="G28" s="19">
-        <f>SUM(G10:G27)</f>
-        <v>9490</v>
+        <v>3871</v>
       </c>
       <c r="H28" s="19"/>
-      <c r="I28" s="20" t="s">
-        <v>9</v>
+      <c r="I28" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total :</t>
+        </is>
       </c>
       <c r="J28" s="20">
-        <f>I26+I27</f>
-        <v>24074160</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K28"/>
     </row>
     <row r="29" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B29" s="9"/>
@@ -7170,10 +7330,13 @@
       <c r="H29" s="24"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
+      <c r="K29"/>
     </row>
     <row r="30" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B30" s="41" t="s">
-        <v>28</v>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">세금계산서 발행 요청일 : 2026-07-27</t>
+        </is>
       </c>
       <c r="C30" s="42"/>
       <c r="D30" s="42"/>
@@ -7185,9 +7348,14 @@
       <c r="J30" s="21" t="s">
         <v>10</v>
       </c>
+      <c r="K30"/>
     </row>
     <row r="31" spans="2:10" ht="45" customHeight="1">
-      <c r="B31" s="44"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">세금계산서 작성일자 : 2026-07-27</t>
+        </is>
+      </c>
       <c r="C31" s="45"/>
       <c r="D31" s="45"/>
       <c r="E31" s="45"/>
@@ -7197,9 +7365,14 @@
       <c r="J31" s="31" t="s">
         <v>11</v>
       </c>
+      <c r="K31"/>
     </row>
     <row r="32" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B32" s="47"/>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">발행 마감 : 오후 4시</t>
+        </is>
+      </c>
       <c r="C32" s="48"/>
       <c r="D32" s="48"/>
       <c r="E32" s="48"/>
@@ -7209,6 +7382,7 @@
       <c r="J32" s="8" t="s">
         <v>12</v>
       </c>
+      <c r="K32"/>
     </row>
     <row r="33" ht="16.5" customHeight="1"/>
     <row r="34" ht="16.5" customHeight="1"/>
@@ -7231,7 +7405,7 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.51181102362204722" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix settlement templates and fitted previews
</commit_message>
<xml_diff>
--- a/settlement-domestic-template.xlsx
+++ b/settlement-domestic-template.xlsx
@@ -32,8 +32,6 @@
     <definedName name="SD">'[3]KVC_출고의뢰 (2)'!$C$19</definedName>
     <definedName name="SE">'[4]KVC_출고의뢰 (2)'!$C$19</definedName>
     <definedName name="출고의뢰">'[3]KVC_출고의뢰 (2)'!$C$19</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'S.T'!$B$1:$K$32</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'S.T (2)'!$B$1:$K$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -6252,9 +6250,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A0B5D11-80F4-4002-A30B-B2D9878D47EF}">
   <sheetPr>
     <tabColor indexed="18"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:K38"/>
+  <dimension ref="B1:J38"/>
   <sheetFormatPr defaultColWidth="9.75" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -6266,8 +6263,7 @@
     <col min="7" max="8" width="15.58203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.58203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="30.58203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="4" style="1" customWidth="1"/>
-    <col min="12" max="16" width="9.75" style="1" customWidth="1"/>
+    <col min="11" max="16" width="9.75" style="1" customWidth="1"/>
     <col min="17" max="20" width="9.75" style="1"/>
     <col min="21" max="37" width="9.75" style="1" customWidth="1"/>
     <col min="38" max="45" width="9.75" style="1"/>
@@ -6285,17 +6281,15 @@
       <c r="F2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">삼원스틸 주식회사</t>
-        </is>
+      <c r="G2" s="52" t="s">
+        <v>22</v>
       </c>
       <c r="H2" s="52"/>
       <c r="I2" s="22" t="s">
         <v>15</v>
       </c>
       <c r="J2" s="23">
-        <v>46230</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="33" customHeight="1">
@@ -6305,7 +6299,9 @@
       <c r="F3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="52"/>
+      <c r="G3" s="52" t="s">
+        <v>23</v>
+      </c>
       <c r="H3" s="52"/>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -6317,7 +6313,9 @@
       <c r="F4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="52"/>
+      <c r="G4" s="52" t="s">
+        <v>24</v>
+      </c>
       <c r="H4" s="52"/>
       <c r="I4" s="52"/>
       <c r="J4" s="52"/>
@@ -6331,7 +6329,9 @@
       <c r="F5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="52"/>
+      <c r="G5" s="52" t="s">
+        <v>25</v>
+      </c>
       <c r="H5" s="52"/>
       <c r="I5" s="52"/>
       <c r="J5" s="52"/>
@@ -6343,10 +6343,8 @@
       <c r="F6" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">260724-7</t>
-        </is>
+      <c r="G6" s="52">
+        <v>8920</v>
       </c>
       <c r="H6" s="52"/>
       <c r="I6" s="52"/>
@@ -6403,66 +6401,41 @@
       <c r="J9" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="K9" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">사진</t>
-        </is>
-      </c>
     </row>
     <row r="10" spans="2:10" ht="24" customHeight="1">
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">254SMO SOLID</t>
-        </is>
-      </c>
-      <c r="C10" s="13">
-        <v>2777</v>
-      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="12"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 925 · VS</t>
-        </is>
-      </c>
-      <c r="G10" s="15">
-        <v>352</v>
-      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="15">
-        <v>0</v>
-      </c>
+      <c r="I10" s="15"/>
       <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="2:10" ht="24" customHeight="1">
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C-276 SOLID</t>
-        </is>
+      <c r="B11" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="C11" s="13">
-        <v>1094</v>
+        <v>4290</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 718 · VS</t>
-        </is>
+      <c r="F11" s="12" t="str">
+        <f>B11</f>
+        <v>Ti 64 TUR</v>
       </c>
       <c r="G11" s="15">
-        <v>742</v>
+        <v>4125</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11" s="16">
+        <f>G11*H11</f>
         <v>0</v>
       </c>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">●</t>
-        </is>
+      <c r="J11" s="37" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="24" customHeight="1">
@@ -6470,100 +6443,63 @@
       <c r="C12" s="13"/>
       <c r="D12" s="12"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · 254 · SOLID</t>
-        </is>
+      <c r="F12" s="12" t="s">
+        <v>32</v>
       </c>
       <c r="G12" s="15">
-        <v>1277</v>
+        <v>66</v>
       </c>
       <c r="H12" s="16"/>
-      <c r="I12" s="16">
-        <v>0</v>
-      </c>
+      <c r="I12" s="16"/>
       <c r="J12" s="37"/>
-      <c r="K12" s="37"/>
     </row>
     <row r="13" spans="2:10" ht="24" customHeight="1">
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="12"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · 254 · AS</t>
-        </is>
+      <c r="F13" s="12" t="s">
+        <v>27</v>
       </c>
       <c r="G13" s="15">
-        <v>1200</v>
+        <v>99</v>
       </c>
       <c r="H13" s="16"/>
-      <c r="I13" s="16">
-        <v>0</v>
-      </c>
+      <c r="I13" s="16"/>
       <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
     </row>
     <row r="14" spans="2:10" ht="24" customHeight="1">
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="12"/>
       <c r="E14" s="11"/>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · sus 304 · SOLID</t>
-        </is>
-      </c>
-      <c r="G14" s="15">
-        <v>95</v>
-      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="15"/>
       <c r="H14" s="26"/>
-      <c r="I14" s="26">
-        <v>0</v>
-      </c>
+      <c r="I14" s="26"/>
       <c r="J14" s="37"/>
-      <c r="K14" s="37"/>
     </row>
     <row r="15" spans="2:10" ht="24" customHeight="1">
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="12"/>
       <c r="E15" s="11"/>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 718 · AS</t>
-        </is>
-      </c>
-      <c r="G15" s="15">
-        <v>200</v>
-      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="15"/>
       <c r="H15" s="16"/>
-      <c r="I15" s="16">
-        <v>0</v>
-      </c>
+      <c r="I15" s="16"/>
       <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
     </row>
     <row r="16" spans="2:10" ht="24" customHeight="1">
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="12"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOSS · 작업중 로스</t>
-        </is>
-      </c>
-      <c r="G16" s="15">
-        <v>5</v>
-      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="16"/>
-      <c r="I16" s="16">
-        <v>0</v>
-      </c>
+      <c r="I16" s="16"/>
       <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="2:10" ht="24" customHeight="1">
       <c r="B17" s="12"/>
@@ -6575,7 +6511,6 @@
       <c r="H17" s="26"/>
       <c r="I17" s="26"/>
       <c r="J17" s="37"/>
-      <c r="K17"/>
     </row>
     <row r="18" spans="2:10" ht="24" customHeight="1">
       <c r="B18" s="12"/>
@@ -6587,7 +6522,6 @@
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="37"/>
-      <c r="K18"/>
     </row>
     <row r="19" spans="2:10" ht="24" customHeight="1">
       <c r="B19" s="12"/>
@@ -6599,7 +6533,6 @@
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="37"/>
-      <c r="K19"/>
     </row>
     <row r="20" spans="2:10" ht="24" customHeight="1">
       <c r="B20" s="12"/>
@@ -6611,7 +6544,6 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="37"/>
-      <c r="K20"/>
     </row>
     <row r="21" spans="2:10" ht="24" customHeight="1">
       <c r="B21" s="12"/>
@@ -6623,7 +6555,6 @@
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="17"/>
-      <c r="K21"/>
     </row>
     <row r="22" spans="2:10" ht="24" customHeight="1">
       <c r="B22" s="12"/>
@@ -6635,7 +6566,6 @@
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
       <c r="J22" s="17"/>
-      <c r="K22"/>
     </row>
     <row r="23" spans="2:10" ht="24" customHeight="1">
       <c r="B23" s="12"/>
@@ -6647,7 +6577,6 @@
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
-      <c r="K23"/>
     </row>
     <row r="24" spans="2:10" ht="24" customHeight="1">
       <c r="B24" s="12"/>
@@ -6659,7 +6588,6 @@
       <c r="H24" s="26"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
-      <c r="K24"/>
     </row>
     <row r="25" spans="2:10" ht="24" customHeight="1">
       <c r="B25" s="12"/>
@@ -6671,7 +6599,6 @@
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
-      <c r="K25"/>
     </row>
     <row r="26" spans="2:10" ht="24" customHeight="1">
       <c r="B26" s="17"/>
@@ -6680,16 +6607,14 @@
       <c r="E26" s="11"/>
       <c r="F26" s="14"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">공급가액 :</t>
-        </is>
+      <c r="H26" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="I26" s="15">
+        <f>SUM(I10:I25)</f>
         <v>0</v>
       </c>
       <c r="J26" s="17"/>
-      <c r="K26"/>
     </row>
     <row r="27" spans="2:10" ht="24" customHeight="1">
       <c r="B27" s="18"/>
@@ -6698,46 +6623,38 @@
       <c r="E27" s="11"/>
       <c r="F27" s="14"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부가세 :</t>
-        </is>
+      <c r="H27" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="I27" s="15">
+        <f>I26*10%</f>
         <v>0</v>
       </c>
       <c r="J27" s="18"/>
-      <c r="K27"/>
     </row>
     <row r="28" spans="2:10" ht="24" customHeight="1">
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total</t>
-        </is>
+      <c r="B28" s="35" t="s">
+        <v>8</v>
       </c>
       <c r="C28" s="34">
-        <v>3871</v>
+        <f>SUM(C10:C27)</f>
+        <v>4290</v>
       </c>
       <c r="D28" s="34"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total</t>
-        </is>
-      </c>
+      <c r="F28" s="32"/>
       <c r="G28" s="19">
-        <v>3871</v>
+        <f>SUM(G10:G27)</f>
+        <v>4290</v>
       </c>
       <c r="H28" s="19"/>
-      <c r="I28" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total :</t>
-        </is>
+      <c r="I28" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="J28" s="20">
+        <f>I26+I27</f>
         <v>0</v>
       </c>
-      <c r="K28"/>
     </row>
     <row r="29" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B29" s="9"/>
@@ -6749,13 +6666,10 @@
       <c r="H29" s="24"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
-      <c r="K29"/>
     </row>
     <row r="30" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B30" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">세금계산서 발행 요청일 : 2026-07-27</t>
-        </is>
+      <c r="B30" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="C30" s="42"/>
       <c r="D30" s="42"/>
@@ -6767,14 +6681,9 @@
       <c r="J30" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="K30"/>
     </row>
     <row r="31" spans="2:10" ht="45" customHeight="1">
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">세금계산서 작성일자 : 2026-07-27</t>
-        </is>
-      </c>
+      <c r="B31" s="44"/>
       <c r="C31" s="45"/>
       <c r="D31" s="45"/>
       <c r="E31" s="45"/>
@@ -6784,14 +6693,9 @@
       <c r="J31" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="K31"/>
     </row>
     <row r="32" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B32" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">발행 마감 : 오후 4시</t>
-        </is>
-      </c>
+      <c r="B32" s="47"/>
       <c r="C32" s="48"/>
       <c r="D32" s="48"/>
       <c r="E32" s="48"/>
@@ -6801,7 +6705,6 @@
       <c r="J32" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K32"/>
     </row>
     <row r="33" ht="16.5" customHeight="1"/>
     <row r="34" ht="16.5" customHeight="1"/>
@@ -6824,7 +6727,7 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.51181102362204722" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -6833,9 +6736,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F648DCA-04E3-49E1-80BE-BA0535619566}">
   <sheetPr>
     <tabColor indexed="18"/>
-    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:K38"/>
+  <dimension ref="B1:J38"/>
   <sheetFormatPr defaultColWidth="9.75" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -6847,8 +6749,7 @@
     <col min="7" max="8" width="15.58203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.58203125" style="1" customWidth="1"/>
     <col min="10" max="10" width="30.58203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="4" style="1" customWidth="1"/>
-    <col min="12" max="16" width="9.75" style="1" customWidth="1"/>
+    <col min="11" max="16" width="9.75" style="1" customWidth="1"/>
     <col min="17" max="20" width="9.75" style="1"/>
     <col min="21" max="37" width="9.75" style="1" customWidth="1"/>
     <col min="38" max="45" width="9.75" style="1"/>
@@ -6866,17 +6767,15 @@
       <c r="F2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">삼원스틸 주식회사</t>
-        </is>
+      <c r="G2" s="52" t="s">
+        <v>22</v>
       </c>
       <c r="H2" s="52"/>
       <c r="I2" s="22" t="s">
         <v>15</v>
       </c>
       <c r="J2" s="23">
-        <v>46230</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="33" customHeight="1">
@@ -6886,7 +6785,9 @@
       <c r="F3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="52"/>
+      <c r="G3" s="52" t="s">
+        <v>23</v>
+      </c>
       <c r="H3" s="52"/>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -6898,7 +6799,9 @@
       <c r="F4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="52"/>
+      <c r="G4" s="52" t="s">
+        <v>24</v>
+      </c>
       <c r="H4" s="52"/>
       <c r="I4" s="52"/>
       <c r="J4" s="52"/>
@@ -6912,7 +6815,9 @@
       <c r="F5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="52"/>
+      <c r="G5" s="52" t="s">
+        <v>25</v>
+      </c>
       <c r="H5" s="52"/>
       <c r="I5" s="52"/>
       <c r="J5" s="52"/>
@@ -6924,10 +6829,8 @@
       <c r="F6" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">260724-7</t>
-        </is>
+      <c r="G6" s="52">
+        <v>8920</v>
       </c>
       <c r="H6" s="52"/>
       <c r="I6" s="52"/>
@@ -6984,179 +6887,134 @@
       <c r="J9" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="K9" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">사진</t>
-        </is>
-      </c>
     </row>
     <row r="10" spans="2:10" ht="24" customHeight="1">
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">254SMO SOLID</t>
-        </is>
-      </c>
-      <c r="C10" s="13">
-        <v>2777</v>
-      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="12"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 925 · VS</t>
-        </is>
-      </c>
-      <c r="G10" s="15">
-        <v>352</v>
-      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="16"/>
-      <c r="I10" s="15">
-        <v>0</v>
-      </c>
+      <c r="I10" s="15"/>
       <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="2:10" ht="24" customHeight="1">
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C-276 SOLID</t>
-        </is>
-      </c>
-      <c r="C11" s="13">
-        <v>1094</v>
-      </c>
+      <c r="B11" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="13"/>
       <c r="D11" s="12"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 718 · VS</t>
-        </is>
-      </c>
-      <c r="G11" s="15">
-        <v>742</v>
-      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="16">
-        <v>0</v>
-      </c>
+      <c r="I11" s="16"/>
       <c r="J11" s="37"/>
-      <c r="K11" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">●</t>
-        </is>
-      </c>
     </row>
     <row r="12" spans="2:10" ht="24" customHeight="1">
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
+      <c r="B12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="13">
+        <v>5200</v>
+      </c>
       <c r="D12" s="12"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · 254 · SOLID</t>
-        </is>
+      <c r="F12" s="12" t="str">
+        <f>B12</f>
+        <v>Ti 64 TUR</v>
       </c>
       <c r="G12" s="15">
-        <v>1277</v>
-      </c>
-      <c r="H12" s="16"/>
+        <v>5060</v>
+      </c>
+      <c r="H12" s="16">
+        <v>3000</v>
+      </c>
       <c r="I12" s="16">
-        <v>0</v>
+        <f>G12*H12</f>
+        <v>15180000</v>
       </c>
       <c r="J12" s="37"/>
-      <c r="K12" s="37"/>
     </row>
     <row r="13" spans="2:10" ht="24" customHeight="1">
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="12"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · 254 · AS</t>
-        </is>
+      <c r="F13" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="G13" s="15">
-        <v>1200</v>
+        <v>140</v>
       </c>
       <c r="H13" s="16"/>
-      <c r="I13" s="16">
-        <v>0</v>
-      </c>
+      <c r="I13" s="16"/>
       <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
     </row>
     <row r="14" spans="2:10" ht="24" customHeight="1">
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="12"/>
       <c r="E14" s="11"/>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STS · sus 304 · SOLID</t>
-        </is>
-      </c>
-      <c r="G14" s="15">
-        <v>95</v>
-      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="15"/>
       <c r="H14" s="26"/>
-      <c r="I14" s="26">
-        <v>0</v>
-      </c>
+      <c r="I14" s="26"/>
       <c r="J14" s="37"/>
-      <c r="K14" s="37"/>
     </row>
     <row r="15" spans="2:10" ht="24" customHeight="1">
-      <c r="B15" s="12"/>
+      <c r="B15" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="C15" s="13"/>
       <c r="D15" s="12"/>
       <c r="E15" s="11"/>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NI · IN 718 · AS</t>
-        </is>
-      </c>
-      <c r="G15" s="15">
-        <v>200</v>
-      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="15"/>
       <c r="H15" s="26"/>
-      <c r="I15" s="26">
-        <v>0</v>
-      </c>
+      <c r="I15" s="26"/>
       <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
     </row>
     <row r="16" spans="2:10" ht="24" customHeight="1">
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
+      <c r="B16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="13">
+        <v>4290</v>
+      </c>
       <c r="D16" s="12"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOSS · 작업중 로스</t>
-        </is>
+      <c r="F16" s="12" t="str">
+        <f>B16</f>
+        <v>Ti 64 TUR</v>
       </c>
       <c r="G16" s="15">
-        <v>5</v>
-      </c>
-      <c r="H16" s="16"/>
+        <v>4191</v>
+      </c>
+      <c r="H16" s="16">
+        <v>1600</v>
+      </c>
       <c r="I16" s="16">
-        <v>0</v>
+        <f>G16*H16</f>
+        <v>6705600</v>
       </c>
       <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="2:10" ht="24" customHeight="1">
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="12"/>
       <c r="E17" s="11"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="15"/>
+      <c r="F17" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="15">
+        <v>99</v>
+      </c>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="37"/>
-      <c r="K17"/>
     </row>
     <row r="18" spans="2:10" ht="24" customHeight="1">
       <c r="B18" s="12"/>
@@ -7168,7 +7026,6 @@
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="37"/>
-      <c r="K18"/>
     </row>
     <row r="19" spans="2:10" ht="24" customHeight="1">
       <c r="B19" s="12"/>
@@ -7180,7 +7037,6 @@
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="37"/>
-      <c r="K19"/>
     </row>
     <row r="20" spans="2:10" ht="24" customHeight="1">
       <c r="B20" s="12"/>
@@ -7192,7 +7048,6 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="37"/>
-      <c r="K20"/>
     </row>
     <row r="21" spans="2:10" ht="24" customHeight="1">
       <c r="B21" s="12"/>
@@ -7204,7 +7059,6 @@
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="17"/>
-      <c r="K21"/>
     </row>
     <row r="22" spans="2:10" ht="24" customHeight="1">
       <c r="B22" s="12"/>
@@ -7216,7 +7070,6 @@
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
       <c r="J22" s="17"/>
-      <c r="K22"/>
     </row>
     <row r="23" spans="2:10" ht="24" customHeight="1">
       <c r="B23" s="12"/>
@@ -7228,7 +7081,6 @@
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
-      <c r="K23"/>
     </row>
     <row r="24" spans="2:10" ht="24" customHeight="1">
       <c r="B24" s="12"/>
@@ -7240,7 +7092,6 @@
       <c r="H24" s="26"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
-      <c r="K24"/>
     </row>
     <row r="25" spans="2:10" ht="24" customHeight="1">
       <c r="B25" s="12"/>
@@ -7252,7 +7103,6 @@
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
-      <c r="K25"/>
     </row>
     <row r="26" spans="2:10" ht="24" customHeight="1">
       <c r="B26" s="17"/>
@@ -7261,16 +7111,14 @@
       <c r="E26" s="11"/>
       <c r="F26" s="14"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">공급가액 :</t>
-        </is>
+      <c r="H26" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="I26" s="15">
-        <v>0</v>
+        <f>SUM(I10:I25)</f>
+        <v>21885600</v>
       </c>
       <c r="J26" s="17"/>
-      <c r="K26"/>
     </row>
     <row r="27" spans="2:10" ht="24" customHeight="1">
       <c r="B27" s="18"/>
@@ -7279,46 +7127,38 @@
       <c r="E27" s="11"/>
       <c r="F27" s="14"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부가세 :</t>
-        </is>
+      <c r="H27" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="I27" s="15">
-        <v>0</v>
+        <f>I26*10%</f>
+        <v>2188560</v>
       </c>
       <c r="J27" s="18"/>
-      <c r="K27"/>
     </row>
     <row r="28" spans="2:10" ht="24" customHeight="1">
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total</t>
-        </is>
+      <c r="B28" s="35" t="s">
+        <v>8</v>
       </c>
       <c r="C28" s="34">
-        <v>3871</v>
+        <f>SUM(C10:C27)</f>
+        <v>9490</v>
       </c>
       <c r="D28" s="34"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total</t>
-        </is>
-      </c>
+      <c r="F28" s="32"/>
       <c r="G28" s="19">
-        <v>3871</v>
+        <f>SUM(G10:G27)</f>
+        <v>9490</v>
       </c>
       <c r="H28" s="19"/>
-      <c r="I28" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total :</t>
-        </is>
+      <c r="I28" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="J28" s="20">
-        <v>0</v>
-      </c>
-      <c r="K28"/>
+        <f>I26+I27</f>
+        <v>24074160</v>
+      </c>
     </row>
     <row r="29" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B29" s="9"/>
@@ -7330,13 +7170,10 @@
       <c r="H29" s="24"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
-      <c r="K29"/>
     </row>
     <row r="30" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B30" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">세금계산서 발행 요청일 : 2026-07-27</t>
-        </is>
+      <c r="B30" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="C30" s="42"/>
       <c r="D30" s="42"/>
@@ -7348,14 +7185,9 @@
       <c r="J30" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="K30"/>
     </row>
     <row r="31" spans="2:10" ht="45" customHeight="1">
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">세금계산서 작성일자 : 2026-07-27</t>
-        </is>
-      </c>
+      <c r="B31" s="44"/>
       <c r="C31" s="45"/>
       <c r="D31" s="45"/>
       <c r="E31" s="45"/>
@@ -7365,14 +7197,9 @@
       <c r="J31" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="K31"/>
     </row>
     <row r="32" spans="2:10" ht="45" customHeight="1" thickBot="1">
-      <c r="B32" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">발행 마감 : 오후 4시</t>
-        </is>
-      </c>
+      <c r="B32" s="47"/>
       <c r="C32" s="48"/>
       <c r="D32" s="48"/>
       <c r="E32" s="48"/>
@@ -7382,7 +7209,6 @@
       <c r="J32" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K32"/>
     </row>
     <row r="33" ht="16.5" customHeight="1"/>
     <row r="34" ht="16.5" customHeight="1"/>
@@ -7405,7 +7231,7 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.51181102362204722" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>